<commit_message>
phase1C: lock controlled dataset scope
</commit_message>
<xml_diff>
--- a/CHECKLIST_TRIEN_KHAI_FULL.xlsx
+++ b/CHECKLIST_TRIEN_KHAI_FULL.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\ssl_detection_xray_v2\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{09207129-1A4B-46C1-B7D5-6D3EF425D170}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5790F303-62CD-4FE9-A75D-210CB7B4C7F8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -2226,7 +2226,7 @@
       </c>
       <c r="B4" s="2">
         <f>COUNTIF(Checklist!$F:$F,"Chưa làm")</f>
-        <v>438</v>
+        <v>428</v>
       </c>
       <c r="D4" s="3" t="s">
         <v>4</v>
@@ -2262,7 +2262,7 @@
       </c>
       <c r="B6" s="2">
         <f>COUNTIF(Checklist!$F:$F,"Hoàn thành")</f>
-        <v>55</v>
+        <v>65</v>
       </c>
       <c r="D6" s="3" t="s">
         <v>10</v>
@@ -2298,7 +2298,7 @@
       </c>
       <c r="B8" s="5">
         <f>IFERROR(B6/B3,0)</f>
-        <v>0.1111111111111111</v>
+        <v>0.13131313131313133</v>
       </c>
       <c r="D8" s="3" t="s">
         <v>16</v>
@@ -2434,7 +2434,7 @@
       </c>
       <c r="C14">
         <f>'Phase Summary'!C4</f>
-        <v>23</v>
+        <v>13</v>
       </c>
       <c r="D14">
         <f>'Phase Summary'!D4</f>
@@ -2442,7 +2442,7 @@
       </c>
       <c r="E14">
         <f>'Phase Summary'!E4</f>
-        <v>28</v>
+        <v>38</v>
       </c>
       <c r="F14">
         <f>'Phase Summary'!F4</f>
@@ -2454,7 +2454,7 @@
       </c>
       <c r="H14" s="6">
         <f>'Phase Summary'!H4</f>
-        <v>0.5490196078431373</v>
+        <v>0.74509803921568629</v>
       </c>
     </row>
     <row r="15" spans="1:8">
@@ -4883,7 +4883,7 @@
         <v>120</v>
       </c>
       <c r="F61" s="10" t="s">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="G61" s="10" t="s">
         <v>52</v>
@@ -4897,7 +4897,7 @@
       <c r="L61" s="10"/>
       <c r="M61" s="10">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="62" spans="1:13" ht="27.6">
@@ -4917,7 +4917,7 @@
         <v>121</v>
       </c>
       <c r="F62" s="10" t="s">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="G62" s="10" t="s">
         <v>52</v>
@@ -4931,7 +4931,7 @@
       <c r="L62" s="10"/>
       <c r="M62" s="10">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="63" spans="1:13" ht="27.6">
@@ -4951,7 +4951,7 @@
         <v>122</v>
       </c>
       <c r="F63" s="10" t="s">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="G63" s="10" t="s">
         <v>52</v>
@@ -4965,7 +4965,7 @@
       <c r="L63" s="10"/>
       <c r="M63" s="10">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="64" spans="1:13" ht="27.6">
@@ -4985,7 +4985,7 @@
         <v>123</v>
       </c>
       <c r="F64" s="10" t="s">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="G64" s="10" t="s">
         <v>52</v>
@@ -4999,7 +4999,7 @@
       <c r="L64" s="10"/>
       <c r="M64" s="10">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="65" spans="1:13" ht="27.6">
@@ -5019,7 +5019,7 @@
         <v>124</v>
       </c>
       <c r="F65" s="10" t="s">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="G65" s="10" t="s">
         <v>52</v>
@@ -5033,7 +5033,7 @@
       <c r="L65" s="10"/>
       <c r="M65" s="10">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="66" spans="1:13" ht="27.6">
@@ -5053,7 +5053,7 @@
         <v>125</v>
       </c>
       <c r="F66" s="10" t="s">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="G66" s="10" t="s">
         <v>63</v>
@@ -5067,7 +5067,7 @@
       <c r="L66" s="10"/>
       <c r="M66" s="10">
         <f t="shared" ref="M66:M129" si="1">IF(F66="Hoàn thành",1,0)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="67" spans="1:13" ht="27.6">
@@ -5087,7 +5087,7 @@
         <v>126</v>
       </c>
       <c r="F67" s="10" t="s">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="G67" s="10" t="s">
         <v>63</v>
@@ -5101,7 +5101,7 @@
       <c r="L67" s="10"/>
       <c r="M67" s="10">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="68" spans="1:13" ht="27.6">
@@ -5121,7 +5121,7 @@
         <v>127</v>
       </c>
       <c r="F68" s="10" t="s">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="G68" s="10" t="s">
         <v>52</v>
@@ -5135,7 +5135,7 @@
       <c r="L68" s="10"/>
       <c r="M68" s="10">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="69" spans="1:13" ht="27.6">
@@ -5155,7 +5155,7 @@
         <v>128</v>
       </c>
       <c r="F69" s="10" t="s">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="G69" s="10" t="s">
         <v>52</v>
@@ -5169,7 +5169,7 @@
       <c r="L69" s="10"/>
       <c r="M69" s="10">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="70" spans="1:13" ht="27.6">
@@ -5189,7 +5189,7 @@
         <v>129</v>
       </c>
       <c r="F70" s="10" t="s">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="G70" s="10" t="s">
         <v>52</v>
@@ -5203,7 +5203,7 @@
       <c r="L70" s="10"/>
       <c r="M70" s="10">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="71" spans="1:13" ht="27.6">
@@ -19854,7 +19854,7 @@
       </c>
       <c r="C4">
         <f>COUNTIFS(Checklist!$B:$B,A4,Checklist!$F:$F,"Chưa làm")</f>
-        <v>23</v>
+        <v>13</v>
       </c>
       <c r="D4">
         <f>COUNTIFS(Checklist!$B:$B,A4,Checklist!$F:$F,"Đang làm")</f>
@@ -19862,7 +19862,7 @@
       </c>
       <c r="E4">
         <f>COUNTIFS(Checklist!$B:$B,A4,Checklist!$F:$F,"Hoàn thành")</f>
-        <v>28</v>
+        <v>38</v>
       </c>
       <c r="F4">
         <f>COUNTIFS(Checklist!$B:$B,A4,Checklist!$F:$F,"Bị chặn")</f>
@@ -19874,7 +19874,7 @@
       </c>
       <c r="H4" s="6">
         <f t="shared" si="0"/>
-        <v>0.5490196078431373</v>
+        <v>0.74509803921568629</v>
       </c>
     </row>
     <row r="5" spans="1:8">

</xml_diff>

<commit_message>
phase1D: document kappa agreement evidence
</commit_message>
<xml_diff>
--- a/CHECKLIST_TRIEN_KHAI_FULL.xlsx
+++ b/CHECKLIST_TRIEN_KHAI_FULL.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\ssl_detection_xray_v2\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5790F303-62CD-4FE9-A75D-210CB7B4C7F8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C88A3FC6-CA18-4D31-8C61-3F2AA2D38875}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -2226,7 +2226,7 @@
       </c>
       <c r="B4" s="2">
         <f>COUNTIF(Checklist!$F:$F,"Chưa làm")</f>
-        <v>428</v>
+        <v>415</v>
       </c>
       <c r="D4" s="3" t="s">
         <v>4</v>
@@ -2262,7 +2262,7 @@
       </c>
       <c r="B6" s="2">
         <f>COUNTIF(Checklist!$F:$F,"Hoàn thành")</f>
-        <v>65</v>
+        <v>78</v>
       </c>
       <c r="D6" s="3" t="s">
         <v>10</v>
@@ -2298,7 +2298,7 @@
       </c>
       <c r="B8" s="5">
         <f>IFERROR(B6/B3,0)</f>
-        <v>0.13131313131313133</v>
+        <v>0.15757575757575756</v>
       </c>
       <c r="D8" s="3" t="s">
         <v>16</v>
@@ -2434,7 +2434,7 @@
       </c>
       <c r="C14">
         <f>'Phase Summary'!C4</f>
-        <v>13</v>
+        <v>0</v>
       </c>
       <c r="D14">
         <f>'Phase Summary'!D4</f>
@@ -2442,7 +2442,7 @@
       </c>
       <c r="E14">
         <f>'Phase Summary'!E4</f>
-        <v>38</v>
+        <v>51</v>
       </c>
       <c r="F14">
         <f>'Phase Summary'!F4</f>
@@ -2454,7 +2454,7 @@
       </c>
       <c r="H14" s="6">
         <f>'Phase Summary'!H4</f>
-        <v>0.74509803921568629</v>
+        <v>1</v>
       </c>
     </row>
     <row r="15" spans="1:8">
@@ -5223,7 +5223,7 @@
         <v>131</v>
       </c>
       <c r="F71" s="10" t="s">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="G71" s="10" t="s">
         <v>63</v>
@@ -5237,7 +5237,7 @@
       <c r="L71" s="10"/>
       <c r="M71" s="10">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="72" spans="1:13" ht="27.6">
@@ -5257,7 +5257,7 @@
         <v>132</v>
       </c>
       <c r="F72" s="10" t="s">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="G72" s="10" t="s">
         <v>63</v>
@@ -5271,7 +5271,7 @@
       <c r="L72" s="10"/>
       <c r="M72" s="10">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="73" spans="1:13" ht="27.6">
@@ -5291,7 +5291,7 @@
         <v>133</v>
       </c>
       <c r="F73" s="10" t="s">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="G73" s="10" t="s">
         <v>63</v>
@@ -5305,7 +5305,7 @@
       <c r="L73" s="10"/>
       <c r="M73" s="10">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="74" spans="1:13" ht="27.6">
@@ -5325,7 +5325,7 @@
         <v>134</v>
       </c>
       <c r="F74" s="10" t="s">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="G74" s="10" t="s">
         <v>63</v>
@@ -5339,7 +5339,7 @@
       <c r="L74" s="10"/>
       <c r="M74" s="10">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="75" spans="1:13" ht="27.6">
@@ -5359,7 +5359,7 @@
         <v>135</v>
       </c>
       <c r="F75" s="10" t="s">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="G75" s="10" t="s">
         <v>63</v>
@@ -5373,7 +5373,7 @@
       <c r="L75" s="10"/>
       <c r="M75" s="10">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="76" spans="1:13" ht="27.6">
@@ -5393,7 +5393,7 @@
         <v>136</v>
       </c>
       <c r="F76" s="10" t="s">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="G76" s="10" t="s">
         <v>52</v>
@@ -5407,7 +5407,7 @@
       <c r="L76" s="10"/>
       <c r="M76" s="10">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="77" spans="1:13" ht="27.6">
@@ -5427,7 +5427,7 @@
         <v>137</v>
       </c>
       <c r="F77" s="10" t="s">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="G77" s="10" t="s">
         <v>63</v>
@@ -5441,7 +5441,7 @@
       <c r="L77" s="10"/>
       <c r="M77" s="10">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="78" spans="1:13" ht="27.6">
@@ -5461,7 +5461,7 @@
         <v>138</v>
       </c>
       <c r="F78" s="10" t="s">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="G78" s="10" t="s">
         <v>63</v>
@@ -5475,7 +5475,7 @@
       <c r="L78" s="10"/>
       <c r="M78" s="10">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="79" spans="1:13" ht="27.6">
@@ -5495,7 +5495,7 @@
         <v>139</v>
       </c>
       <c r="F79" s="10" t="s">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="G79" s="10" t="s">
         <v>63</v>
@@ -5509,7 +5509,7 @@
       <c r="L79" s="10"/>
       <c r="M79" s="10">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="80" spans="1:13" ht="27.6">
@@ -5529,7 +5529,7 @@
         <v>140</v>
       </c>
       <c r="F80" s="10" t="s">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="G80" s="10" t="s">
         <v>63</v>
@@ -5543,7 +5543,7 @@
       <c r="L80" s="10"/>
       <c r="M80" s="10">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="81" spans="1:13" ht="27.6">
@@ -5563,7 +5563,7 @@
         <v>141</v>
       </c>
       <c r="F81" s="10" t="s">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="G81" s="10" t="s">
         <v>52</v>
@@ -5577,7 +5577,7 @@
       <c r="L81" s="10"/>
       <c r="M81" s="10">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="82" spans="1:13" ht="27.6">
@@ -5597,7 +5597,7 @@
         <v>142</v>
       </c>
       <c r="F82" s="10" t="s">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="G82" s="10" t="s">
         <v>52</v>
@@ -5611,7 +5611,7 @@
       <c r="L82" s="10"/>
       <c r="M82" s="10">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="83" spans="1:13" ht="27.6">
@@ -5631,7 +5631,7 @@
         <v>143</v>
       </c>
       <c r="F83" s="10" t="s">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="G83" s="10" t="s">
         <v>52</v>
@@ -5645,7 +5645,7 @@
       <c r="L83" s="10"/>
       <c r="M83" s="10">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="84" spans="1:13" ht="27.6">
@@ -19854,7 +19854,7 @@
       </c>
       <c r="C4">
         <f>COUNTIFS(Checklist!$B:$B,A4,Checklist!$F:$F,"Chưa làm")</f>
-        <v>13</v>
+        <v>0</v>
       </c>
       <c r="D4">
         <f>COUNTIFS(Checklist!$B:$B,A4,Checklist!$F:$F,"Đang làm")</f>
@@ -19862,7 +19862,7 @@
       </c>
       <c r="E4">
         <f>COUNTIFS(Checklist!$B:$B,A4,Checklist!$F:$F,"Hoàn thành")</f>
-        <v>38</v>
+        <v>51</v>
       </c>
       <c r="F4">
         <f>COUNTIFS(Checklist!$B:$B,A4,Checklist!$F:$F,"Bị chặn")</f>
@@ -19874,7 +19874,7 @@
       </c>
       <c r="H4" s="6">
         <f t="shared" si="0"/>
-        <v>0.74509803921568629</v>
+        <v>1</v>
       </c>
     </row>
     <row r="5" spans="1:8">

</xml_diff>

<commit_message>
phase2A: validate DICOM availability and bbox boundaries
</commit_message>
<xml_diff>
--- a/CHECKLIST_TRIEN_KHAI_FULL.xlsx
+++ b/CHECKLIST_TRIEN_KHAI_FULL.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\ssl_detection_xray_v2\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C88A3FC6-CA18-4D31-8C61-3F2AA2D38875}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9AC21191-9E08-4C57-829A-5847C3F45687}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -2226,7 +2226,7 @@
       </c>
       <c r="B4" s="2">
         <f>COUNTIF(Checklist!$F:$F,"Chưa làm")</f>
-        <v>415</v>
+        <v>399</v>
       </c>
       <c r="D4" s="3" t="s">
         <v>4</v>
@@ -2262,7 +2262,7 @@
       </c>
       <c r="B6" s="2">
         <f>COUNTIF(Checklist!$F:$F,"Hoàn thành")</f>
-        <v>78</v>
+        <v>94</v>
       </c>
       <c r="D6" s="3" t="s">
         <v>10</v>
@@ -2298,7 +2298,7 @@
       </c>
       <c r="B8" s="5">
         <f>IFERROR(B6/B3,0)</f>
-        <v>0.15757575757575756</v>
+        <v>0.1898989898989899</v>
       </c>
       <c r="D8" s="3" t="s">
         <v>16</v>
@@ -2467,7 +2467,7 @@
       </c>
       <c r="C15">
         <f>'Phase Summary'!C5</f>
-        <v>115</v>
+        <v>99</v>
       </c>
       <c r="D15">
         <f>'Phase Summary'!D5</f>
@@ -2475,7 +2475,7 @@
       </c>
       <c r="E15">
         <f>'Phase Summary'!E5</f>
-        <v>0</v>
+        <v>16</v>
       </c>
       <c r="F15">
         <f>'Phase Summary'!F5</f>
@@ -2487,7 +2487,7 @@
       </c>
       <c r="H15" s="6">
         <f>'Phase Summary'!H5</f>
-        <v>0</v>
+        <v>0.1391304347826087</v>
       </c>
     </row>
     <row r="16" spans="1:8">
@@ -5665,7 +5665,7 @@
         <v>145</v>
       </c>
       <c r="F84" s="10" t="s">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="G84" s="10" t="s">
         <v>63</v>
@@ -5679,7 +5679,7 @@
       <c r="L84" s="10"/>
       <c r="M84" s="10">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="85" spans="1:13" ht="27.6">
@@ -5699,7 +5699,7 @@
         <v>146</v>
       </c>
       <c r="F85" s="10" t="s">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="G85" s="10" t="s">
         <v>63</v>
@@ -5713,7 +5713,7 @@
       <c r="L85" s="10"/>
       <c r="M85" s="10">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="86" spans="1:13" ht="27.6">
@@ -5733,7 +5733,7 @@
         <v>147</v>
       </c>
       <c r="F86" s="10" t="s">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="G86" s="10" t="s">
         <v>63</v>
@@ -5747,7 +5747,7 @@
       <c r="L86" s="10"/>
       <c r="M86" s="10">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="87" spans="1:13" ht="27.6">
@@ -5767,7 +5767,7 @@
         <v>148</v>
       </c>
       <c r="F87" s="10" t="s">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="G87" s="10" t="s">
         <v>63</v>
@@ -5781,7 +5781,7 @@
       <c r="L87" s="10"/>
       <c r="M87" s="10">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="88" spans="1:13" ht="27.6">
@@ -5801,7 +5801,7 @@
         <v>149</v>
       </c>
       <c r="F88" s="10" t="s">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="G88" s="10" t="s">
         <v>63</v>
@@ -5815,7 +5815,7 @@
       <c r="L88" s="10"/>
       <c r="M88" s="10">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="89" spans="1:13" ht="27.6">
@@ -5835,7 +5835,7 @@
         <v>150</v>
       </c>
       <c r="F89" s="10" t="s">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="G89" s="10" t="s">
         <v>63</v>
@@ -5849,7 +5849,7 @@
       <c r="L89" s="10"/>
       <c r="M89" s="10">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="90" spans="1:13" ht="27.6">
@@ -5869,7 +5869,7 @@
         <v>151</v>
       </c>
       <c r="F90" s="10" t="s">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="G90" s="10" t="s">
         <v>52</v>
@@ -5883,7 +5883,7 @@
       <c r="L90" s="10"/>
       <c r="M90" s="10">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="91" spans="1:13" ht="27.6">
@@ -5903,7 +5903,7 @@
         <v>152</v>
       </c>
       <c r="F91" s="10" t="s">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="G91" s="10" t="s">
         <v>52</v>
@@ -5917,7 +5917,7 @@
       <c r="L91" s="10"/>
       <c r="M91" s="10">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="92" spans="1:13" ht="27.6">
@@ -5937,7 +5937,7 @@
         <v>153</v>
       </c>
       <c r="F92" s="10" t="s">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="G92" s="10" t="s">
         <v>63</v>
@@ -5951,7 +5951,7 @@
       <c r="L92" s="10"/>
       <c r="M92" s="10">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="93" spans="1:13" ht="27.6">
@@ -5971,7 +5971,7 @@
         <v>154</v>
       </c>
       <c r="F93" s="10" t="s">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="G93" s="10" t="s">
         <v>63</v>
@@ -5985,7 +5985,7 @@
       <c r="L93" s="10"/>
       <c r="M93" s="10">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="94" spans="1:13" ht="27.6">
@@ -6005,7 +6005,7 @@
         <v>155</v>
       </c>
       <c r="F94" s="10" t="s">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="G94" s="10" t="s">
         <v>63</v>
@@ -6019,7 +6019,7 @@
       <c r="L94" s="10"/>
       <c r="M94" s="10">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="95" spans="1:13" ht="27.6">
@@ -6039,7 +6039,7 @@
         <v>156</v>
       </c>
       <c r="F95" s="10" t="s">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="G95" s="10" t="s">
         <v>63</v>
@@ -6053,7 +6053,7 @@
       <c r="L95" s="10"/>
       <c r="M95" s="10">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="96" spans="1:13" ht="27.6">
@@ -6073,7 +6073,7 @@
         <v>157</v>
       </c>
       <c r="F96" s="10" t="s">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="G96" s="10" t="s">
         <v>52</v>
@@ -6087,7 +6087,7 @@
       <c r="L96" s="10"/>
       <c r="M96" s="10">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="97" spans="1:13" ht="27.6">
@@ -6107,7 +6107,7 @@
         <v>158</v>
       </c>
       <c r="F97" s="10" t="s">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="G97" s="10" t="s">
         <v>52</v>
@@ -6121,7 +6121,7 @@
       <c r="L97" s="10"/>
       <c r="M97" s="10">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="98" spans="1:13" ht="27.6">
@@ -6141,7 +6141,7 @@
         <v>159</v>
       </c>
       <c r="F98" s="10" t="s">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="G98" s="10" t="s">
         <v>52</v>
@@ -6155,7 +6155,7 @@
       <c r="L98" s="10"/>
       <c r="M98" s="10">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="99" spans="1:13" ht="27.6">
@@ -6175,7 +6175,7 @@
         <v>160</v>
       </c>
       <c r="F99" s="10" t="s">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="G99" s="10" t="s">
         <v>52</v>
@@ -6189,7 +6189,7 @@
       <c r="L99" s="10"/>
       <c r="M99" s="10">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="100" spans="1:13" ht="27.6">
@@ -19887,7 +19887,7 @@
       </c>
       <c r="C5">
         <f>COUNTIFS(Checklist!$B:$B,A5,Checklist!$F:$F,"Chưa làm")</f>
-        <v>115</v>
+        <v>99</v>
       </c>
       <c r="D5">
         <f>COUNTIFS(Checklist!$B:$B,A5,Checklist!$F:$F,"Đang làm")</f>
@@ -19895,7 +19895,7 @@
       </c>
       <c r="E5">
         <f>COUNTIFS(Checklist!$B:$B,A5,Checklist!$F:$F,"Hoàn thành")</f>
-        <v>0</v>
+        <v>16</v>
       </c>
       <c r="F5">
         <f>COUNTIFS(Checklist!$B:$B,A5,Checklist!$F:$F,"Bị chặn")</f>
@@ -19907,7 +19907,7 @@
       </c>
       <c r="H5" s="6">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>0.1391304347826087</v>
       </c>
     </row>
     <row r="6" spans="1:8">

</xml_diff>

<commit_message>
docs: update phase2B handoff and checklist
</commit_message>
<xml_diff>
--- a/CHECKLIST_TRIEN_KHAI_FULL.xlsx
+++ b/CHECKLIST_TRIEN_KHAI_FULL.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\ssl_detection_xray_v2\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9AC21191-9E08-4C57-829A-5847C3F45687}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F767C65C-3E04-4648-9ADA-3154C7F8F888}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -2226,7 +2226,7 @@
       </c>
       <c r="B4" s="2">
         <f>COUNTIF(Checklist!$F:$F,"Chưa làm")</f>
-        <v>399</v>
+        <v>387</v>
       </c>
       <c r="D4" s="3" t="s">
         <v>4</v>
@@ -2262,7 +2262,7 @@
       </c>
       <c r="B6" s="2">
         <f>COUNTIF(Checklist!$F:$F,"Hoàn thành")</f>
-        <v>94</v>
+        <v>106</v>
       </c>
       <c r="D6" s="3" t="s">
         <v>10</v>
@@ -2298,7 +2298,7 @@
       </c>
       <c r="B8" s="5">
         <f>IFERROR(B6/B3,0)</f>
-        <v>0.1898989898989899</v>
+        <v>0.21414141414141413</v>
       </c>
       <c r="D8" s="3" t="s">
         <v>16</v>
@@ -2467,7 +2467,7 @@
       </c>
       <c r="C15">
         <f>'Phase Summary'!C5</f>
-        <v>99</v>
+        <v>87</v>
       </c>
       <c r="D15">
         <f>'Phase Summary'!D5</f>
@@ -2475,7 +2475,7 @@
       </c>
       <c r="E15">
         <f>'Phase Summary'!E5</f>
-        <v>16</v>
+        <v>28</v>
       </c>
       <c r="F15">
         <f>'Phase Summary'!F5</f>
@@ -2487,7 +2487,7 @@
       </c>
       <c r="H15" s="6">
         <f>'Phase Summary'!H5</f>
-        <v>0.1391304347826087</v>
+        <v>0.24347826086956523</v>
       </c>
     </row>
     <row r="16" spans="1:8">
@@ -6209,7 +6209,7 @@
         <v>162</v>
       </c>
       <c r="F100" s="10" t="s">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="G100" s="10" t="s">
         <v>63</v>
@@ -6223,7 +6223,7 @@
       <c r="L100" s="10"/>
       <c r="M100" s="10">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="101" spans="1:13" ht="27.6">
@@ -6243,7 +6243,7 @@
         <v>163</v>
       </c>
       <c r="F101" s="10" t="s">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="G101" s="10" t="s">
         <v>63</v>
@@ -6257,7 +6257,7 @@
       <c r="L101" s="10"/>
       <c r="M101" s="10">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="102" spans="1:13" ht="27.6">
@@ -6277,7 +6277,7 @@
         <v>164</v>
       </c>
       <c r="F102" s="10" t="s">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="G102" s="10" t="s">
         <v>63</v>
@@ -6291,7 +6291,7 @@
       <c r="L102" s="10"/>
       <c r="M102" s="10">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="103" spans="1:13" ht="27.6">
@@ -6311,7 +6311,7 @@
         <v>165</v>
       </c>
       <c r="F103" s="10" t="s">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="G103" s="10" t="s">
         <v>63</v>
@@ -6325,7 +6325,7 @@
       <c r="L103" s="10"/>
       <c r="M103" s="10">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="104" spans="1:13" ht="27.6">
@@ -6345,7 +6345,7 @@
         <v>166</v>
       </c>
       <c r="F104" s="10" t="s">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="G104" s="10" t="s">
         <v>63</v>
@@ -6359,7 +6359,7 @@
       <c r="L104" s="10"/>
       <c r="M104" s="10">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="105" spans="1:13" ht="27.6">
@@ -6379,7 +6379,7 @@
         <v>167</v>
       </c>
       <c r="F105" s="10" t="s">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="G105" s="10" t="s">
         <v>63</v>
@@ -6393,7 +6393,7 @@
       <c r="L105" s="10"/>
       <c r="M105" s="10">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="106" spans="1:13" ht="27.6">
@@ -6413,7 +6413,7 @@
         <v>168</v>
       </c>
       <c r="F106" s="10" t="s">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="G106" s="10" t="s">
         <v>63</v>
@@ -6427,7 +6427,7 @@
       <c r="L106" s="10"/>
       <c r="M106" s="10">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="107" spans="1:13" ht="27.6">
@@ -6447,7 +6447,7 @@
         <v>169</v>
       </c>
       <c r="F107" s="10" t="s">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="G107" s="10" t="s">
         <v>63</v>
@@ -6461,7 +6461,7 @@
       <c r="L107" s="10"/>
       <c r="M107" s="10">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="108" spans="1:13" ht="27.6">
@@ -6481,7 +6481,7 @@
         <v>170</v>
       </c>
       <c r="F108" s="10" t="s">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="G108" s="10" t="s">
         <v>63</v>
@@ -6495,7 +6495,7 @@
       <c r="L108" s="10"/>
       <c r="M108" s="10">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="109" spans="1:13" ht="27.6">
@@ -6515,7 +6515,7 @@
         <v>171</v>
       </c>
       <c r="F109" s="10" t="s">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="G109" s="10" t="s">
         <v>52</v>
@@ -6529,7 +6529,7 @@
       <c r="L109" s="10"/>
       <c r="M109" s="10">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="110" spans="1:13" ht="27.6">
@@ -6549,7 +6549,7 @@
         <v>172</v>
       </c>
       <c r="F110" s="10" t="s">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="G110" s="10" t="s">
         <v>52</v>
@@ -6563,7 +6563,7 @@
       <c r="L110" s="10"/>
       <c r="M110" s="10">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="111" spans="1:13" ht="27.6">
@@ -6583,7 +6583,7 @@
         <v>173</v>
       </c>
       <c r="F111" s="10" t="s">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="G111" s="10" t="s">
         <v>52</v>
@@ -6597,7 +6597,7 @@
       <c r="L111" s="10"/>
       <c r="M111" s="10">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="112" spans="1:13" ht="27.6">
@@ -19887,7 +19887,7 @@
       </c>
       <c r="C5">
         <f>COUNTIFS(Checklist!$B:$B,A5,Checklist!$F:$F,"Chưa làm")</f>
-        <v>99</v>
+        <v>87</v>
       </c>
       <c r="D5">
         <f>COUNTIFS(Checklist!$B:$B,A5,Checklist!$F:$F,"Đang làm")</f>
@@ -19895,7 +19895,7 @@
       </c>
       <c r="E5">
         <f>COUNTIFS(Checklist!$B:$B,A5,Checklist!$F:$F,"Hoàn thành")</f>
-        <v>16</v>
+        <v>28</v>
       </c>
       <c r="F5">
         <f>COUNTIFS(Checklist!$B:$B,A5,Checklist!$F:$F,"Bị chặn")</f>
@@ -19907,7 +19907,7 @@
       </c>
       <c r="H5" s="6">
         <f t="shared" si="0"/>
-        <v>0.1391304347826087</v>
+        <v>0.24347826086956523</v>
       </c>
     </row>
     <row r="6" spans="1:8">

</xml_diff>

<commit_message>
phase2C: decide framework and COCO planning protocol
</commit_message>
<xml_diff>
--- a/CHECKLIST_TRIEN_KHAI_FULL.xlsx
+++ b/CHECKLIST_TRIEN_KHAI_FULL.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\ssl_detection_xray_v2\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F767C65C-3E04-4648-9ADA-3154C7F8F888}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{722D5090-6DDA-46AC-9235-E1EDB014D092}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -2226,7 +2226,7 @@
       </c>
       <c r="B4" s="2">
         <f>COUNTIF(Checklist!$F:$F,"Chưa làm")</f>
-        <v>387</v>
+        <v>376</v>
       </c>
       <c r="D4" s="3" t="s">
         <v>4</v>
@@ -2262,7 +2262,7 @@
       </c>
       <c r="B6" s="2">
         <f>COUNTIF(Checklist!$F:$F,"Hoàn thành")</f>
-        <v>106</v>
+        <v>117</v>
       </c>
       <c r="D6" s="3" t="s">
         <v>10</v>
@@ -2298,7 +2298,7 @@
       </c>
       <c r="B8" s="5">
         <f>IFERROR(B6/B3,0)</f>
-        <v>0.21414141414141413</v>
+        <v>0.23636363636363636</v>
       </c>
       <c r="D8" s="3" t="s">
         <v>16</v>
@@ -2467,7 +2467,7 @@
       </c>
       <c r="C15">
         <f>'Phase Summary'!C5</f>
-        <v>87</v>
+        <v>76</v>
       </c>
       <c r="D15">
         <f>'Phase Summary'!D5</f>
@@ -2475,7 +2475,7 @@
       </c>
       <c r="E15">
         <f>'Phase Summary'!E5</f>
-        <v>28</v>
+        <v>39</v>
       </c>
       <c r="F15">
         <f>'Phase Summary'!F5</f>
@@ -2487,7 +2487,7 @@
       </c>
       <c r="H15" s="6">
         <f>'Phase Summary'!H5</f>
-        <v>0.24347826086956523</v>
+        <v>0.33913043478260868</v>
       </c>
     </row>
     <row r="16" spans="1:8">
@@ -6617,7 +6617,7 @@
         <v>175</v>
       </c>
       <c r="F112" s="10" t="s">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="G112" s="10" t="s">
         <v>52</v>
@@ -6631,7 +6631,7 @@
       <c r="L112" s="10"/>
       <c r="M112" s="10">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="113" spans="1:13" ht="27.6">
@@ -6651,7 +6651,7 @@
         <v>176</v>
       </c>
       <c r="F113" s="10" t="s">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="G113" s="10" t="s">
         <v>52</v>
@@ -6665,7 +6665,7 @@
       <c r="L113" s="10"/>
       <c r="M113" s="10">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="114" spans="1:13" ht="27.6">
@@ -6685,7 +6685,7 @@
         <v>177</v>
       </c>
       <c r="F114" s="10" t="s">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="G114" s="10" t="s">
         <v>52</v>
@@ -6699,7 +6699,7 @@
       <c r="L114" s="10"/>
       <c r="M114" s="10">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="115" spans="1:13" ht="27.6">
@@ -6719,7 +6719,7 @@
         <v>178</v>
       </c>
       <c r="F115" s="10" t="s">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="G115" s="10" t="s">
         <v>52</v>
@@ -6733,7 +6733,7 @@
       <c r="L115" s="10"/>
       <c r="M115" s="10">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="116" spans="1:13" ht="27.6">
@@ -6753,7 +6753,7 @@
         <v>179</v>
       </c>
       <c r="F116" s="10" t="s">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="G116" s="10" t="s">
         <v>52</v>
@@ -6767,7 +6767,7 @@
       <c r="L116" s="10"/>
       <c r="M116" s="10">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="117" spans="1:13" ht="27.6">
@@ -6787,7 +6787,7 @@
         <v>180</v>
       </c>
       <c r="F117" s="10" t="s">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="G117" s="10" t="s">
         <v>52</v>
@@ -6801,7 +6801,7 @@
       <c r="L117" s="10"/>
       <c r="M117" s="10">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="118" spans="1:13" ht="27.6">
@@ -6821,7 +6821,7 @@
         <v>181</v>
       </c>
       <c r="F118" s="10" t="s">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="G118" s="10" t="s">
         <v>63</v>
@@ -6835,7 +6835,7 @@
       <c r="L118" s="10"/>
       <c r="M118" s="10">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="119" spans="1:13" ht="27.6">
@@ -6855,7 +6855,7 @@
         <v>182</v>
       </c>
       <c r="F119" s="10" t="s">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="G119" s="10" t="s">
         <v>63</v>
@@ -6869,7 +6869,7 @@
       <c r="L119" s="10"/>
       <c r="M119" s="10">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="120" spans="1:13" ht="27.6">
@@ -6889,7 +6889,7 @@
         <v>183</v>
       </c>
       <c r="F120" s="10" t="s">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="G120" s="10" t="s">
         <v>63</v>
@@ -6903,7 +6903,7 @@
       <c r="L120" s="10"/>
       <c r="M120" s="10">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="121" spans="1:13" ht="27.6">
@@ -6923,7 +6923,7 @@
         <v>184</v>
       </c>
       <c r="F121" s="10" t="s">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="G121" s="10" t="s">
         <v>52</v>
@@ -6937,7 +6937,7 @@
       <c r="L121" s="10"/>
       <c r="M121" s="10">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="122" spans="1:13" ht="27.6">
@@ -6957,7 +6957,7 @@
         <v>185</v>
       </c>
       <c r="F122" s="10" t="s">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="G122" s="10" t="s">
         <v>52</v>
@@ -6971,7 +6971,7 @@
       <c r="L122" s="10"/>
       <c r="M122" s="10">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="123" spans="1:13" ht="27.6">
@@ -19887,7 +19887,7 @@
       </c>
       <c r="C5">
         <f>COUNTIFS(Checklist!$B:$B,A5,Checklist!$F:$F,"Chưa làm")</f>
-        <v>87</v>
+        <v>76</v>
       </c>
       <c r="D5">
         <f>COUNTIFS(Checklist!$B:$B,A5,Checklist!$F:$F,"Đang làm")</f>
@@ -19895,7 +19895,7 @@
       </c>
       <c r="E5">
         <f>COUNTIFS(Checklist!$B:$B,A5,Checklist!$F:$F,"Hoàn thành")</f>
-        <v>28</v>
+        <v>39</v>
       </c>
       <c r="F5">
         <f>COUNTIFS(Checklist!$B:$B,A5,Checklist!$F:$F,"Bị chặn")</f>
@@ -19907,7 +19907,7 @@
       </c>
       <c r="H5" s="6">
         <f t="shared" si="0"/>
-        <v>0.24347826086956523</v>
+        <v>0.33913043478260868</v>
       </c>
     </row>
     <row r="6" spans="1:8">

</xml_diff>